<commit_message>
Funktionsmatrix: Umsetzungsstand Phase 4 Teil 1, Zoom-Screenshot um Seitenmitte
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): leeres Dokument mit wählbarem Format; Erstellung aus Office/CAD offen</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Seiten aus einer anderen PDF einfügen; Mehrfachauswahl von Dateien offen</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Seitenbereich in neue Datei extrahieren; Aufteilen nach Lesezeichen oder Seitenzahl offen</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Seite vor/zurück per Befehl; Drag &amp; Drop in Miniaturen offen</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Seitenlabels werden angezeigt; Bearbeiten offen</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Lesezeichen anzeigen und anspringen; Bearbeiten offen</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Eigenschaften und Metadaten anzeigen; Bearbeiten offen</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3549,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Seitenleiste mit Miniaturen und Lesezeichen</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 1): Statusleiste mit Pfad, Seitenformat und Zoom</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kopieren, Einfügen, Duplizieren, Einrasten mit Umschalttaste; Umsetzungsstand in der Funktionsmatrix
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -3971,7 +3971,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 4, Teil 1): Seitenleiste mit Miniaturen und Lesezeichen</t>
+          <t>Teilweise (Phase 4, Teil 2): Seitenleiste mit Miniaturen, Lesezeichen und Suche; Markierungsliste unten</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2): Suche über alle Seiten, Trefferliste, Hervorhebung, F3</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Kontextmenüs für Miniaturen und Markierungen</t>
         </is>
       </c>
     </row>
@@ -7327,7 +7327,7 @@
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7398,7 +7398,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7469,7 +7469,7 @@
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7607,7 +7607,7 @@
       <c r="N102" s="2" t="inlineStr"/>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7674,7 @@
       <c r="N103" s="2" t="inlineStr"/>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7741,7 +7741,7 @@
       <c r="N104" s="2" t="inlineStr"/>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7812,7 @@
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -8021,7 +8021,7 @@
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -8159,7 +8159,7 @@
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -8360,7 +8360,7 @@
       <c r="N113" s="2" t="inlineStr"/>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -8494,7 +8494,7 @@
       <c r="N115" s="2" t="inlineStr"/>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Bereich hervorheben; an Textauswahl gebunden offen</t>
         </is>
       </c>
     </row>
@@ -9976,7 +9976,7 @@
       <c r="N137" s="2" t="inlineStr"/>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2): Klick, Strg+Klick, Strg+A</t>
         </is>
       </c>
     </row>
@@ -10039,7 +10039,7 @@
       <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Verschieben und Skalieren; Drehen offen</t>
         </is>
       </c>
     </row>
@@ -10177,7 +10177,7 @@
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Kopieren und Einfügen (Strg+C, Strg+V); Ausschneiden und an Position einfügen offen</t>
         </is>
       </c>
     </row>
@@ -10244,7 +10244,7 @@
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2): Strg+D</t>
         </is>
       </c>
     </row>
@@ -10508,7 +10508,7 @@
       <c r="N145" s="2" t="inlineStr"/>
       <c r="O145" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Vordergrund und Hintergrund über Kontextmenü</t>
         </is>
       </c>
     </row>
@@ -10646,7 +10646,7 @@
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Farbe, Linienbreite, Deckkraft, Füllung, Text, Kommentar</t>
         </is>
       </c>
     </row>
@@ -10784,7 +10784,7 @@
       </c>
       <c r="O149" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2)</t>
         </is>
       </c>
     </row>
@@ -11060,7 +11060,7 @@
       <c r="N153" s="2" t="inlineStr"/>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2): Umschalttaste beim Zeichnen</t>
         </is>
       </c>
     </row>
@@ -11738,7 +11738,7 @@
       <c r="N163" s="2" t="inlineStr"/>
       <c r="O163" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 2): Eckpunkte von Linien, Polygonen und Messungen ziehen</t>
         </is>
       </c>
     </row>
@@ -11809,7 +11809,7 @@
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Liste aller Markierungen des Dokuments</t>
         </is>
       </c>
     </row>
@@ -11876,7 +11876,7 @@
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Seite, Art, Wert, Text, Maßstab, Autor, Datum</t>
         </is>
       </c>
     </row>
@@ -11943,7 +11943,7 @@
       </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Sortieren und Filtern; Gruppieren offen</t>
         </is>
       </c>
     </row>
@@ -12278,7 +12278,7 @@
       </c>
       <c r="O171" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Summen je Messart in der Liste</t>
         </is>
       </c>
     </row>
@@ -12345,7 +12345,7 @@
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): CSV-Export für Excel; XLSX offen</t>
         </is>
       </c>
     </row>
@@ -12885,7 +12885,7 @@
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -12960,7 +12960,7 @@
       </c>
       <c r="O181" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -13031,7 +13031,7 @@
       <c r="N182" s="2" t="inlineStr"/>
       <c r="O182" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13106,7 @@
       </c>
       <c r="O183" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1): Fläche mit Umfang</t>
         </is>
       </c>
     </row>
@@ -13587,7 +13587,7 @@
       <c r="N190" s="2" t="inlineStr"/>
       <c r="O190" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -13926,7 +13926,7 @@
       <c r="N195" s="2" t="inlineStr"/>
       <c r="O195" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -14052,7 +14052,7 @@
       <c r="N197" s="2" t="inlineStr"/>
       <c r="O197" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Summen in der Liste und für ausgewählte Messungen</t>
         </is>
       </c>
     </row>
@@ -14328,7 +14328,7 @@
       </c>
       <c r="O201" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1): übliche Maßstäbe 1:1 bis 1:2000 je Seite</t>
         </is>
       </c>
     </row>
@@ -14395,7 +14395,7 @@
       </c>
       <c r="O202" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1)</t>
         </is>
       </c>
     </row>
@@ -14592,7 +14592,7 @@
       </c>
       <c r="O205" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): m, cm, mm</t>
         </is>
       </c>
     </row>
@@ -14726,7 +14726,7 @@
       <c r="N207" s="2" t="inlineStr"/>
       <c r="O207" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 1): Mengenliste mit Summen und CSV-Export</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flächen mit Ausschnitten (Abzüge), Drucken und Ausschnitte in Matrix und Anleitung
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -2705,7 +2705,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 4, Teil 2): Drucken über den Windows-Druckdialog mit Seitenauswahl, eingepasst</t>
         </is>
       </c>
     </row>
@@ -13382,7 +13382,7 @@
       <c r="N187" s="2" t="inlineStr"/>
       <c r="O187" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 1): Ausschnitte per Rechtsklick auf eine Fläche</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Volumen, Wandflächen und Excel-Export der Mengenliste
Messungen können eine Tiefe (Fläche, ergibt Volumen) oder Höhe (Länge,
Polylänge, Umfang, ergibt Wandfläche) bekommen, über das Kontextmenü.
Die Liste summiert beides; der Export schreibt XLSX mit Summenblatt,
CSV bleibt wählbar. Listenmodell und XLSX-Schreiber liegen jetzt in
Egle360.Pdf und sind getestet.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -12345,7 +12345,7 @@
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 5, Teil 1): CSV-Export für Excel; XLSX offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): XLSX mit Summenblatt, alternativ CSV</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
       <c r="N184" s="2" t="inlineStr"/>
       <c r="O184" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): Tiefe je Fläche, Volumen in m³</t>
         </is>
       </c>
     </row>
@@ -13248,7 +13248,7 @@
       </c>
       <c r="O185" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): Höhe je Länge, Polylänge oder Umfang, Wandfläche in m²</t>
         </is>
       </c>
     </row>
@@ -14726,7 +14726,7 @@
       <c r="N207" s="2" t="inlineStr"/>
       <c r="O207" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 5, Teil 1): Mengenliste mit Summen und CSV-Export</t>
+          <t>Teilweise (Phase 5, Teil 2): Mengenliste mit Summen, Volumen und Wandflächen, Export als XLSX oder CSV</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Radius und Durchmesser messen
Zwei neue Messwerkzeuge mit Kreis und Kreisfläche in der Liste.
Werte, die sich nicht sinnvoll addieren lassen (Winkel, Bemaßung,
Radius, Durchmesser), bleiben aus den Summen heraus.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -13654,7 +13654,7 @@
       <c r="N191" s="2" t="inlineStr"/>
       <c r="O191" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): mit Kreisfläche in der Liste</t>
         </is>
       </c>
     </row>
@@ -13721,7 +13721,7 @@
       <c r="N192" s="2" t="inlineStr"/>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): mit Kreisfläche in der Liste</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Status, Sperren und Einheitspreise für Markierungen
Status (Offen bis Freigegeben) mit Person und Zeitpunkt, Sperre gegen
Verschieben, Ändern und Löschen, Einheitspreis je Messung mit
Gesamtpreis und Kostensumme in Liste, CSV und XLSX. Gespeichert in den
EGLE360-Daten der Anmerkung, die Sperre zusätzlich als Locked-Flag.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -10713,7 +10713,7 @@
       <c r="N148" s="2" t="inlineStr"/>
       <c r="O148" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): Sperren und Entsperren, im PDF zusätzlich mit Locked-Flag</t>
         </is>
       </c>
     </row>
@@ -12144,7 +12144,7 @@
       <c r="N169" s="2" t="inlineStr"/>
       <c r="O169" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 2): sechs feste Status mit Person und Zeitpunkt; eigene Statusmodelle offen</t>
         </is>
       </c>
     </row>
@@ -14793,7 +14793,7 @@
       <c r="N208" s="2" t="inlineStr"/>
       <c r="O208" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 2): Einheitspreis je Messung, Gesamtpreis und Kostensumme in Liste und Export; Preislisten je Werkzeug offen</t>
         </is>
       </c>
     </row>
@@ -14994,7 +14994,7 @@
       <c r="N211" s="2" t="inlineStr"/>
       <c r="O211" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 2): Status Geprüft und Freigegeben mit Person und Zeitpunkt, Sperren; eigener Freigabeablauf offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ausrichten, Darstellung übertragen, Markierungen ausblenden
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -10378,7 +10378,7 @@
       <c r="N143" s="2" t="inlineStr"/>
       <c r="O143" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): sechs Ausrichtungen und Verteilen, bezogen auf die angezeigte Seitendrehung</t>
         </is>
       </c>
     </row>
@@ -10575,7 +10575,7 @@
       <c r="N146" s="2" t="inlineStr"/>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 2): Darstellung kopieren und einfügen (Strg+Umschalt+C/V)</t>
         </is>
       </c>
     </row>
@@ -12475,7 +12475,7 @@
       <c r="N174" s="2" t="inlineStr"/>
       <c r="O174" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 2): alle Markierungen ein- und ausblenden; nach Art oder Autor offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Text hervorheben, unterstreichen und durchstreichen entlang der Textzeilen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -8494,7 +8494,7 @@
       <c r="N115" s="2" t="inlineStr"/>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 4, Teil 2): Bereich hervorheben; an Textauswahl gebunden offen</t>
+          <t>Umgesetzt (Phase 4, Teil 3): folgt den Textzeilen im aufgezogenen Bereich, ohne Text als Rechteck</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8561,7 @@
       <c r="N116" s="2" t="inlineStr"/>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 3): je Textzeile, als PDF-Underline mit QuadPoints</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       <c r="N117" s="2" t="inlineStr"/>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 4, Teil 3): je Textzeile, als PDF-StrikeOut mit QuadPoints</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Werkzeugbibliothek mit Werkzeugsätzen, Suche, Favoriten, Import und Export
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -15061,7 +15061,7 @@
       <c r="N212" s="2" t="inlineStr"/>
       <c r="O212" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 3): Werkzeugsätze in der Seitenleiste, Werkzeug aus Markierung speichern, bleibt beim Zeichnen aktiv</t>
         </is>
       </c>
     </row>
@@ -15195,7 +15195,7 @@
       </c>
       <c r="O214" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 3): Import und Export im eigenen Format e360-tools (JSON); BTX-Import offen</t>
         </is>
       </c>
     </row>
@@ -15258,7 +15258,7 @@
       <c r="N215" s="2" t="inlineStr"/>
       <c r="O215" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 3): Suche nach Name, Satz und Art; Favoriten zuerst</t>
         </is>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
       </c>
       <c r="O216" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 3): Grundausstattung Planprüfung und Mengen Hochbau ohne Preise; weitere Gewerke offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planverwaltung mit Planliste, Indexverlauf und Übernahme der Markierungen; Version 0.7.0
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -15459,7 +15459,7 @@
       <c r="N218" s="2" t="inlineStr"/>
       <c r="O218" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 3): Planliste je Projektordner mit Nummer, Bezeichnung, Index, Datum, Verfasser, Gewerk, Geschoss, Gebäude, Bauabschnitt, Status, Freigabe; Excel-Export</t>
         </is>
       </c>
     </row>
@@ -15530,7 +15530,7 @@
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 3): Muster im Seitentext und im Dateinamen; Plankopf-Region und OCR offen</t>
         </is>
       </c>
     </row>
@@ -15601,7 +15601,7 @@
       </c>
       <c r="O220" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 3): neue Indizes nach Plannummer einsortieren, mehrere Dateien auf einmal, Markierungen und Maßstäbe übernehmen</t>
         </is>
       </c>
     </row>
@@ -15664,7 +15664,7 @@
       <c r="N221" s="2" t="inlineStr"/>
       <c r="O221" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 5, Teil 3): jeder Index bleibt als eigene Datei erhalten und lässt sich öffnen</t>
         </is>
       </c>
     </row>
@@ -15873,7 +15873,7 @@
       </c>
       <c r="O224" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 5, Teil 3): Vorschlagsliste mit Gewerkkürzeln, frei änderbar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Markierungen drehen, Planstände vergleichen mit Überlagerung und Änderungswolken, Planverwaltung ohne Auswahllisten
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -10039,7 +10039,7 @@
       <c r="N138" s="2" t="inlineStr"/>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 4, Teil 2): Verschieben und Skalieren; Drehen offen</t>
+          <t>Umgesetzt (Phase 5, Teil 3): Verschieben, Skalieren, Drehen in 90-Grad-Schritten für alle Arten, beliebige Winkel für Punktformen</t>
         </is>
       </c>
     </row>
@@ -15940,7 +15940,7 @@
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6, Teil 1): Seitenweiser Vergleich zweier Stände, Änderungen als Wolken im neuen Stand; stapelweise offen</t>
         </is>
       </c>
     </row>
@@ -16003,7 +16003,7 @@
       <c r="N226" s="2" t="inlineStr"/>
       <c r="O226" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6, Teil 1): Überlagerung rot (alt), blau (neu), grau (gleich); Ebenen und Transparenz offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stapelverarbeitung: Stempel und Maßstab für viele PDF-Dateien
BatchRunner mit Fortschritt, Protokoll, Abbruch und Fortsetzen über bereits
erledigte Kopien. Fenster aus Dokumentansicht und Planverwaltung erreichbar;
Ergebnis standardmäßig als Kopien im Zielordner.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -8900,7 +8900,7 @@
       <c r="N121" s="2" t="inlineStr"/>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Umgesetzt (Phase 6): Stempel auf erste oder alle Seiten vieler Dateien, Ecke wählbar, als Kopien oder in den Originalen</t>
         </is>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="O248" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Stapellauf mit Fortschritt, Protokoll, Abbruch und Fortsetzen über bereits erledigte Kopien; bisher Schritte Stempel und Maßstab</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plansatz vergleichen: alle Pläne gegen den vorherigen Index, Bericht und Wolken
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -15802,7 +15802,7 @@
       <c r="N223" s="2" t="inlineStr"/>
       <c r="O223" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Änderungsbericht je Plan und Index aus dem Plansatzvergleich (Excel)</t>
         </is>
       </c>
     </row>
@@ -15940,7 +15940,7 @@
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 6, Teil 1): Seitenweiser Vergleich zweier Stände, Änderungen als Wolken im neuen Stand; stapelweise offen</t>
+          <t>Umgesetzt (Phase 6): Seitenweiser Vergleich zweier Stände, Änderungen als Wolken im neuen Stand, auch für ganze Plansätze</t>
         </is>
       </c>
     </row>
@@ -16070,7 +16070,7 @@
       </c>
       <c r="O227" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 6, Teil 1): Verschiebung wird automatisch erkannt und ausgeglichen; Drehung, Maßstab und manuelle Ausrichtung offen</t>
+          <t>Offen</t>
         </is>
       </c>
     </row>
@@ -16141,7 +16141,7 @@
       </c>
       <c r="O228" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Verschiebung wird beim Vergleich automatisch erkannt und ausgeglichen; Drehung und Maßstab noch nicht</t>
         </is>
       </c>
     </row>
@@ -16212,7 +16212,7 @@
       </c>
       <c r="O229" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): ganzer Plansatz der Planverwaltung, je Plan aktueller gegen vorherigen Index; freie Ordnervergleiche offen</t>
         </is>
       </c>
     </row>
@@ -16417,7 +16417,7 @@
       <c r="N232" s="2" t="inlineStr"/>
       <c r="O232" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Änderungsbericht als Excel-Mappe (je Plan und je Bereich), Wolken in die neuen Stände; PDF-Bericht und Aufgaben offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stapelverarbeitung: Kopf- und Fußzeile, Seiten drehen, Markierungen einbrennen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U3Ukx2hXXYYuHcvsESmy4u
</commit_message>
<xml_diff>
--- a/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
+++ b/docs/phase1/EGLE360_PLAN_Funktionsmatrix.xlsx
@@ -2149,7 +2149,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Kopf- und Fußzeile mit Dateiname, Seite, Seitenzahl und Datum über die Stapelverarbeitung, fest im Seiteninhalt; Entfernen und Bearbeiten offen</t>
         </is>
       </c>
     </row>
@@ -10851,7 +10851,7 @@
       <c r="N150" s="2" t="inlineStr"/>
       <c r="O150" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Teilweise (Phase 6): Einbrennen über die Stapelverarbeitung, Maßstab bleibt erhalten; Rückwandlung offen</t>
         </is>
       </c>
     </row>
@@ -17497,7 +17497,7 @@
       </c>
       <c r="O248" s="2" t="inlineStr">
         <is>
-          <t>Teilweise (Phase 6): Stapellauf mit Fortschritt, Protokoll, Abbruch und Fortsetzen über bereits erledigte Kopien; bisher Schritte Stempel und Maßstab</t>
+          <t>Teilweise (Phase 6): Stapellauf mit Fortschritt, Protokoll, Abbruch und Fortsetzen über bereits erledigte Kopien; Schritte Stempel, Maßstab, Kopf- und Fußzeile, Seiten drehen und Markierungen einbrennen</t>
         </is>
       </c>
     </row>

</xml_diff>